<commit_message>
Graph 1 gemacht Emulsion
</commit_message>
<xml_diff>
--- a/Emulsionspoly/Tabelle MEsswerte.xlsx
+++ b/Emulsionspoly/Tabelle MEsswerte.xlsx
@@ -1,20 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dokumente\Uni laptop\Chemie\Poly\Emulsionspoly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C217600E-519A-41E6-9BF1-8B9280DBC80C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A9C303C-A5C4-46DB-8AE8-F33F2B70C8F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{25867DC9-E48D-4029-A39F-4AFAE13D5DF5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{25867DC9-E48D-4029-A39F-4AFAE13D5DF5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Diagramm1" sheetId="2" r:id="rId1"/>
+    <sheet name="Tabelle1" sheetId="1" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Tabelle1!$A$6:$A$18</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Tabelle1!$H$5</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">Tabelle1!$H$6:$H$18</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -177,6 +183,1990 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Tabelle1!$H$6:$H$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>12.591445141555806</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.896776349716303</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.322046755262841</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9.1264786676926644</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10.219787339302359</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9.2196284352253333</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8.3784245408557272</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8.8048281521715275</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9.9860245870663498</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10.179079664857662</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11.815573269687656</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>19.664162430051352</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>59.994024776179877</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0AE0-4D77-AF8C-1EA3923E3CBA}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="580916447"/>
+        <c:axId val="580915487"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="580916447"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="580915487"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="580915487"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="580916447"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Umsatz-Zeit-Diagramm</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout>
+        <c:manualLayout>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.39065311372906608"/>
+          <c:y val="2.4055889217894741E-2"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="de-DE"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Tabelle1!$H$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Umsatz [%]</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>Tabelle1!$A$6:$A$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>150</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>180</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Tabelle1!$H$6:$H$18</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>12.591445141555806</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>8.896776349716303</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10.322046755262841</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9.1264786676926644</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>10.219787339302359</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>9.2196284352253333</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>8.3784245408557272</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8.8048281521715275</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9.9860245870663498</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10.179079664857662</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11.815573269687656</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>19.664162430051352</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>59.994024776179877</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-711D-481C-BE0E-7154FA85C98D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="596230751"/>
+        <c:axId val="596232671"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="596230751"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE" sz="1100" b="1" i="0" baseline="0"/>
+                  <a:t>Reaktionsdauer in [min]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="596232671"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="596232671"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="de-DE" sz="1100" b="1" i="0" strike="noStrike" baseline="0"/>
+                  <a:t>Umsatz in [%]</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="de-DE"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="de-DE"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="596230751"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="de-DE"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.7" r="0.7" t="0.78740157499999996" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{6D1BE5A8-2A8E-4E09-9CAE-ED316870FAEF}">
+  <sheetPr/>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</chartsheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:absoluteAnchor>
+    <xdr:pos x="0" y="0"/>
+    <xdr:ext cx="9305774" cy="6017381"/>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Diagramm 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{52E803C0-694F-3F45-C43F-E9B2E82D2B2E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks noGrp="1"/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:absoluteAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2291601</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>34738</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>190500</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>67236</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="13" name="Diagramm 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F65730F6-BBE1-BCF6-E6FD-C7C013224D11}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -505,7 +2495,7 @@
     <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="7.140625" bestFit="1" customWidth="1"/>
@@ -610,7 +2600,7 @@
         <v>8.3999999999999631E-2</v>
       </c>
       <c r="H6">
-        <f>(G6*$L$6*100)/($J$6*(1+$K$6/$J$6)*E6)</f>
+        <f>(G6*$L$6*100)/($J$6*(1+($K$6/$J$6))*E6)</f>
         <v>12.591445141555806</v>
       </c>
       <c r="J6">
@@ -651,7 +2641,7 @@
         <v>5.7000000000000384E-2</v>
       </c>
       <c r="H7">
-        <f>(G7*$L$6*100)/($J$6*(1+$K$6/$J$6)*E7)</f>
+        <f t="shared" ref="H7:H18" si="2">(G7*$L$6*100)/($J$6*(1+($K$6/$J$6))*E7)</f>
         <v>8.896776349716303</v>
       </c>
     </row>
@@ -680,7 +2670,7 @@
         <v>6.9900000000000517E-2</v>
       </c>
       <c r="H8">
-        <f t="shared" ref="H8:H18" si="2">(G8*$L$6*100)/($J$6*(1+$K$6/$J$6)*E8)</f>
+        <f t="shared" si="2"/>
         <v>10.322046755262841</v>
       </c>
     </row>
@@ -977,5 +2967,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Tabelle überarbeitet und Argumentiert
</commit_message>
<xml_diff>
--- a/Emulsionspoly/Tabelle MEsswerte.xlsx
+++ b/Emulsionspoly/Tabelle MEsswerte.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dokumente\Uni laptop\Chemie\Poly\Emulsionspoly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E487475-185C-4AF8-BCAC-1F7943EAC93E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{001A5569-66FA-4F9A-B371-FF34C4BB71DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{25867DC9-E48D-4029-A39F-4AFAE13D5DF5}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="16305" activeTab="1" xr2:uid="{25867DC9-E48D-4029-A39F-4AFAE13D5DF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Diagramm1" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
   <si>
     <t>Nr.</t>
   </si>
@@ -118,6 +118,24 @@
   </si>
   <si>
     <t>Umsatz [%]</t>
+  </si>
+  <si>
+    <t>v_Br in %/min</t>
+  </si>
+  <si>
+    <t>0.0002</t>
+  </si>
+  <si>
+    <t>0.0004</t>
+  </si>
+  <si>
+    <t>0.0003</t>
+  </si>
+  <si>
+    <t>0.0005</t>
+  </si>
+  <si>
+    <t>0.0008</t>
   </si>
 </sst>
 </file>
@@ -2490,7 +2508,7 @@
     <col min="6" max="6" width="43.140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="35.140625" customWidth="1"/>
     <col min="10" max="10" width="6.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="7.140625" bestFit="1" customWidth="1"/>
@@ -2557,6 +2575,9 @@
       <c r="H5" t="s">
         <v>26</v>
       </c>
+      <c r="I5" t="s">
+        <v>27</v>
+      </c>
       <c r="J5" t="s">
         <v>21</v>
       </c>
@@ -2598,6 +2619,9 @@
         <f>(G6*$L$6*100)/($J$6*(1+($K$6/$J$6))*E6)</f>
         <v>12.591445141555806</v>
       </c>
+      <c r="I6" t="s">
+        <v>28</v>
+      </c>
       <c r="J6">
         <v>11.83</v>
       </c>
@@ -2639,6 +2663,9 @@
         <f t="shared" ref="H7:H18" si="2">(G7*$L$6*100)/($J$6*(1+($K$6/$J$6))*E7)</f>
         <v>8.896776349716303</v>
       </c>
+      <c r="I7" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8">
@@ -2668,6 +2695,9 @@
         <f t="shared" si="2"/>
         <v>10.322046755262841</v>
       </c>
+      <c r="I8" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9">
@@ -2697,6 +2727,9 @@
         <f t="shared" si="2"/>
         <v>9.1264786676926644</v>
       </c>
+      <c r="I9" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10">
@@ -2726,6 +2759,9 @@
         <f t="shared" si="2"/>
         <v>10.219787339302359</v>
       </c>
+      <c r="I10" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -2755,6 +2791,9 @@
         <f t="shared" si="2"/>
         <v>9.2196284352253333</v>
       </c>
+      <c r="I11" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -2783,6 +2822,9 @@
       <c r="H12">
         <f t="shared" si="2"/>
         <v>8.3784245408557272</v>
+      </c>
+      <c r="I12" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>